<commit_message>
3PG parms moved to single UI file
</commit_message>
<xml_diff>
--- a/Templates/f_E_coef.xlsx
+++ b/Templates/f_E_coef.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob.osullivan\OneDrive - Forest Research\Turbines and trees\CCWoP\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://forestresearch-my.sharepoint.com/personal/jacob_osullivan_forestresearch_gov_uk/Documents/Turbines and trees/CCWoP/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10A039E-92E3-4154-94B9-BDBB877F6E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="268" documentId="11_F25DC773A252ABDACC1048B0D15C56F85BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{191ECD8F-64B2-4D52-8D68-3249F3CA7912}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -86,13 +86,13 @@
     <t>a4</t>
   </si>
   <si>
+    <t>spp</t>
+  </si>
+  <si>
     <t>Scots_Pine</t>
   </si>
   <si>
     <t>Sitka_Spruce</t>
-  </si>
-  <si>
-    <t>spp</t>
   </si>
   <si>
     <t>f_E</t>
@@ -105,10 +105,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -134,9 +141,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -417,7 +425,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -426,275 +433,338 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D2" s="2">
+        <v>0.126</v>
+      </c>
+      <c r="E2" s="2">
+        <v>7.9100000000000004E-2</v>
+      </c>
+      <c r="F2" s="2">
+        <v>-1.2200000000000001E-2</v>
+      </c>
+      <c r="G2" s="2">
+        <v>9.8900000000000008E-4</v>
+      </c>
+      <c r="H2" s="2">
+        <v>-2.7500000000000001E-5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="2">
+        <v>-1.8500000000000001E-3</v>
+      </c>
+      <c r="E3" s="2">
+        <v>6.2700000000000006E-2</v>
+      </c>
+      <c r="F3" s="2">
+        <v>-5.5199999999999997E-4</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2.6100000000000001E-5</v>
+      </c>
+      <c r="H3" s="1">
         <v>0</v>
       </c>
-      <c r="E1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2">
+        <v>7.22E-2</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.26400000000000001</v>
+      </c>
+      <c r="G4" s="2">
+        <v>-9.9699999999999997E-2</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="1">
-        <v>0.12550529999999999</v>
-      </c>
-      <c r="E2" s="1">
-        <v>7.9110609999999998E-2</v>
-      </c>
-      <c r="F2" s="1">
-        <v>-1.2173969999999999E-2</v>
-      </c>
-      <c r="G2" s="1">
-        <v>9.8886739999999996E-4</v>
-      </c>
-      <c r="H2" s="1">
-        <v>-2.749263E-5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="D5" s="2">
+        <v>0.113</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.13800000000000001</v>
+      </c>
+      <c r="F5" s="2">
+        <v>-2.41E-2</v>
+      </c>
+      <c r="G5" s="2">
+        <v>6.5500000000000003E-2</v>
+      </c>
+      <c r="H5" s="2">
+        <v>-7.7299999999999995E-5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="1">
-        <v>-1.8501139999999999E-3</v>
-      </c>
-      <c r="E3" s="1">
-        <v>6.2660170000000001E-2</v>
-      </c>
-      <c r="F3" s="1">
-        <v>-5.5241619999999998E-4</v>
-      </c>
-      <c r="G3" s="1">
-        <v>2.6055509999999999E-5</v>
-      </c>
-      <c r="H3">
+      <c r="D6" s="2">
+        <v>6.5500000000000003E-2</v>
+      </c>
+      <c r="E6" s="2">
+        <v>8.4500000000000006E-2</v>
+      </c>
+      <c r="F6" s="2">
+        <v>9.75E-3</v>
+      </c>
+      <c r="G6" s="2">
+        <v>-4.4499999999999997E-4</v>
+      </c>
+      <c r="H6" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="1">
-        <v>7.2214650000000005E-2</v>
-      </c>
-      <c r="E4" s="1">
-        <v>0.21171693999999999</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0.26354071000000001</v>
-      </c>
-      <c r="G4" s="1">
-        <v>-9.9735950000000004E-2</v>
-      </c>
-      <c r="H4" s="1">
+      <c r="D7" s="2">
+        <v>0.125</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0.38600000000000001</v>
+      </c>
+      <c r="F7" s="2">
+        <v>-7.2500000000000004E-3</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1.35E-2</v>
+      </c>
+      <c r="H7" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0.1128803</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0.13783139999999999</v>
-      </c>
-      <c r="F5" s="1">
-        <v>-2.4068889999999999E-2</v>
-      </c>
-      <c r="G5" s="1">
-        <v>6.55287009E-2</v>
-      </c>
-      <c r="H5" s="1">
-        <v>-7.7324819999999997E-5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B11" s="1">
+        <v>4</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="2">
+        <v>4.47</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="1">
-        <v>6.55287009E-2</v>
-      </c>
-      <c r="E6" s="1">
-        <v>8.4521816E-2</v>
-      </c>
-      <c r="F6" s="1">
-        <v>9.7538376000000006E-3</v>
-      </c>
-      <c r="G6" s="1">
-        <v>-4.4453279999999998E-4</v>
-      </c>
-      <c r="H6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0.12530286199999999</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0.38619093199999999</v>
-      </c>
-      <c r="F7" s="1">
-        <v>-7.2512729999999999E-3</v>
-      </c>
-      <c r="G7" s="1">
-        <v>1.3542422E-2</v>
-      </c>
-      <c r="H7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="B13" s="1">
+        <v>0.531227267</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="1">
+        <v>0.33044188200000002</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11">
-        <v>4</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="2">
+        <v>0.30299999999999999</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="1">
-        <f>D5+E5*$B$11+F5*POWER($B$11,2)+G5*POWER($B$11,3)</f>
-        <v>4.4729405175999997</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B13">
-        <f>D6+E6*$B$11+F6*POWER($B$11,2)+G6*POWER($B$11,3)</f>
-        <v>0.53122726730000003</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="B17" s="1">
+        <v>0.24161945900000001</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B14">
-        <f>D7+E7*$B$13+F7*POWER($B$13,2)+G7*POWER($B$13,3)</f>
-        <v>0.33044188218535075</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>6</v>
-      </c>
-      <c r="B16" s="1">
-        <f>D2+E2*$B$11+F2*POWER($B$11,2)+G2*POWER($B$11,3)+H2*POWER($B$11,4)</f>
-        <v>0.30341362032000002</v>
-      </c>
-      <c r="C16" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17">
-        <f>D3+E3*$B$11+F3*POWER($B$11,2)+G3*POWER($B$11,3)+H3*POWER($B$11,4)</f>
-        <v>0.24161945943999999</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18">
-        <f>D4+E4*$B$17+F4*POWER($B$17,2)+G4*POWER($B$17,3)+H4*POWER($B$17,4)</f>
-        <v>0.13734823064813795</v>
-      </c>
+      <c r="B18" s="1">
+        <v>0.13734823099999999</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>